<commit_message>
test: correct dynamic array URI expectations from native Excel evidence
Excel for Mac 16.113.4 repairs the uppercase URI previously required by the generated-metadata assertion. A single-attribute lowercase control opens without repair. Correct the strict expectation and synthetic fixture, and retain read/byte-preservation coverage for uppercase, lowercase and mixed source variants. The implementation correction follows separately.
</commit_message>
<xml_diff>
--- a/Tests/SwiftSheetsTests/Fixtures/interop/consumer-contract.xlsx
+++ b/Tests/SwiftSheetsTests/Fixtures/interop/consumer-contract.xlsx
@@ -195,14 +195,14 @@
   <futureMetadata name="XLDAPR" count="2">
     <bk>
       <extLst>
-        <ext uri="{BDBB8CDC-FA1E-496E-A857-3C3F30C029C3}">
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
-        <ext uri="{BDBB8CDC-FA1E-496E-A857-3C3F30C029C3}">
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="0" fCollapsed="0"/>
         </ext>
       </extLst>

</xml_diff>